<commit_message>
Milestone 2 – Template Identification
</commit_message>
<xml_diff>
--- a/data/fixtures/1830-pse-sample.xlsx
+++ b/data/fixtures/1830-pse-sample.xlsx
@@ -8,7 +8,16 @@
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Process" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="PM Est" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Process" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pipe Eng" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Pipe Des" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Elect" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="I&amp;C" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Sched" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Staff Plan" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Dates" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,19 +445,33 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Sample Client</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -459,56 +482,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Discipline</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Deliverable</t>
+          <t>FEL-1</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Activity Name</t>
+          <t>FEL-2</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Qty</t>
+          <t>FEL-3</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Engineer Hrs</t>
+          <t>FEL-4</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
-        <is>
-          <t>Designer Hrs</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Checker Hrs</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>PM Hrs</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Total Hrs</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -517,152 +520,764 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Project Services</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
           <t>Project Services Estimate</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Develop - Project Services Estimate (PSE)</t>
-        </is>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
-      </c>
-      <c r="F2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I2" t="n">
-        <v>23</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>1830 sample line</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Process</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>PFD</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Develop - PFD</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>40</v>
-      </c>
-      <c r="F3" t="n">
-        <v>20</v>
-      </c>
-      <c r="G3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H3" t="n">
-        <v>5</v>
-      </c>
-      <c r="I3" t="n">
-        <v>75</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Process</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>P&amp;ID</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Develop - P&amp;ID</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>80</v>
-      </c>
-      <c r="F4" t="n">
-        <v>40</v>
-      </c>
-      <c r="G4" t="n">
-        <v>20</v>
-      </c>
-      <c r="H4" t="n">
-        <v>8</v>
-      </c>
-      <c r="I4" t="n">
-        <v>148</v>
-      </c>
-      <c r="J4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>I&amp;C</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Preliminary Datasheets</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Develop - Preliminary Datasheets</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>30</v>
-      </c>
-      <c r="F5" t="n">
-        <v>25</v>
-      </c>
-      <c r="G5" t="n">
-        <v>8</v>
-      </c>
-      <c r="H5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" t="n">
-        <v>65</v>
-      </c>
-      <c r="J5" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Sample</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Discipline</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Activity Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Engineer Hrs</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Designer Hrs</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Checker Hrs</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>PM Hrs</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Total Hrs</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Project Services</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Project Services Estimate</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Develop - Project Services Estimate (PSE)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>23</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1830 sample line</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PFD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Develop - PFD</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>75</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Discipline</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Activity Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Engineer Hrs</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Designer Hrs</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Checker Hrs</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>PM Hrs</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Total Hrs</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Project Services</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Project Services Estimate</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Develop - Project Services Estimate (PSE)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>23</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1830 sample line</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PFD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Develop - PFD</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>75</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Discipline</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Activity Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Engineer Hrs</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Designer Hrs</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Checker Hrs</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>PM Hrs</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Total Hrs</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Project Services</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Project Services Estimate</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Develop - Project Services Estimate (PSE)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>23</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1830 sample line</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PFD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Develop - PFD</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>75</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Discipline</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Activity Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Engineer Hrs</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Designer Hrs</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Checker Hrs</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>PM Hrs</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Total Hrs</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Project Services</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Project Services Estimate</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Develop - Project Services Estimate (PSE)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>23</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1830 sample line</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PFD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Develop - PFD</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>75</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Discipline</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Activity Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Engineer Hrs</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Designer Hrs</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Checker Hrs</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>PM Hrs</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Total Hrs</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Project Services</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Project Services Estimate</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Develop - Project Services Estimate (PSE)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>23</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1830 sample line</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PFD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Develop - PFD</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>75</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Milestone 3 – Estimate Line Item Architecture
</commit_message>
<xml_diff>
--- a/data/fixtures/1830-pse-sample.xlsx
+++ b/data/fixtures/1830-pse-sample.xlsx
@@ -482,36 +482,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Discipline</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Deliverable</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>FEL-1</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>FEL-2</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>FEL-3</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>FEL-4</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -520,26 +525,144 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Project Services Estimate</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
+          <t>Project Services</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Project Services Estimate (PSE)</t>
+        </is>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
         <v>25</v>
       </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Sample</t>
-        </is>
-      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1830 PM Est sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Engineering Management</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kick-Off Meeting</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PFD Development</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>P&amp;ID Development</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>80</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>153</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Milestone 3A – Civil/Structural interpreter
</commit_message>
<xml_diff>
--- a/data/fixtures/1830-pse-sample.xlsx
+++ b/data/fixtures/1830-pse-sample.xlsx
@@ -15,9 +15,10 @@
     <sheet name="Pipe Des" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Elect" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="I&amp;C" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Sched" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Staff Plan" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Dates" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Civil Str" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Sched" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Staff Plan" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Dates" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,12 +37,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -56,8 +63,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,6 +484,19 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1398,9 +1419,350 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>1830 Sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Discipline</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Civil/Structural</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Short Form – Task Description</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ENGR HRS</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DESIGN HRS</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>HVE ENGR HRS</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>HVE DESIGN HRS</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Project Investigations</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Geotechnical Report Review</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Studies / Calculations</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Foundation Design Calculations</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" t="n">
+        <v>20</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>General / Building Drawings</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Demo Sketches</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>25</v>
+      </c>
+      <c r="E11" t="n">
+        <v>16</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Platform Sketches</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>16</v>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Project Control</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>99</v>
+      </c>
+      <c r="E16" t="n">
+        <v>53</v>
+      </c>
+      <c r="F16" t="n">
+        <v>14</v>
+      </c>
+      <c r="G16" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" t="n">
+        <v>174</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>